<commit_message>
docs: complete Toolshop test documentation
</commit_message>
<xml_diff>
--- a/testcases/Toolshop_测试用例.xlsx
+++ b/testcases/Toolshop_测试用例.xlsx
@@ -9,13 +9,13 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="16570" windowHeight="12600"/>
+    <workbookView windowWidth="17010" windowHeight="11480"/>
   </bookViews>
   <sheets>
     <sheet name="测试用例" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">测试用例!$A$1:$E$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">测试用例!$A$1:$E$32</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="226">
   <si>
     <t>用例编号</t>
   </si>
@@ -64,6 +64,9 @@
     <t>执行状态</t>
   </si>
   <si>
+    <t>备注</t>
+  </si>
+  <si>
     <t>TC001</t>
   </si>
   <si>
@@ -85,7 +88,10 @@
     <t>1. 点击搜索框；2. 输入一个能在商品列表中找到的商品关键词；3. 执行搜索；4. 查看搜索结果。</t>
   </si>
   <si>
-    <t>未执行</t>
+    <t>搜索 Pliers 后，页面先显示 26 个商品，随后更新为 4 个商品；刷新并重新搜索后现象一致，最终显示的 4 个商品名称均包含 Pliers。</t>
+  </si>
+  <si>
+    <t>通过（Pass）</t>
   </si>
   <si>
     <t>TC002</t>
@@ -103,6 +109,9 @@
     <t>1. 点击搜索框；2. 输入一个确认不存在于商品信息中的关键词；3. 执行搜索；4. 查看页面提示和商品列表。</t>
   </si>
   <si>
+    <t>搜索关键词 xyznonexistent123 后，页面显示 0 products found，未展示匹配商品，页面正常响应。</t>
+  </si>
+  <si>
     <t>TC003</t>
   </si>
   <si>
@@ -121,6 +130,12 @@
     <t>1. 保持搜索框为空；2. 点击搜索按钮或按 Enter；3. 观察页面是否报错、是否显示商品列表或提示。</t>
   </si>
   <si>
+    <t>点击 Search 后，搜索框内文字自动清空；在搜索框为空的情况下再次点击 Search，页面无明显变化。</t>
+  </si>
+  <si>
+    <t>待进一步确认</t>
+  </si>
+  <si>
     <t>TC004</t>
   </si>
   <si>
@@ -133,6 +148,9 @@
     <t>1. 在搜索框输入一个可匹配商品的关键词；2. 在关键词前后各添加空格；3. 执行搜索；4. 检查返回结果。</t>
   </si>
   <si>
+    <t>输入前后带空格的关键词 Pliers 并执行搜索后，最终显示正确的 4 个匹配商品。</t>
+  </si>
+  <si>
     <t>TC005</t>
   </si>
   <si>
@@ -145,6 +163,9 @@
     <t>1. 搜索第一个关键词并记录结果；2. 清空搜索框；3. 输入另一个不同关键词；4. 再次搜索；5. 检查结果是否更新。</t>
   </si>
   <si>
+    <t>先搜索 Pliers，再将关键词更换为 Hammer 并执行搜索，页面能够显示与 Hammer 相关的商品。</t>
+  </si>
+  <si>
     <t>TC006</t>
   </si>
   <si>
@@ -163,6 +184,9 @@
     <t>1. 在商品列表中选择一个商品；2. 点击商品名称、图片或详情入口；3. 查看打开的详情页及其商品信息。</t>
   </si>
   <si>
+    <t>点击商品后，商品详情页正常打开，商品名称、价格、图片及加入购物车按钮均正常显示。</t>
+  </si>
+  <si>
     <t>TC007</t>
   </si>
   <si>
@@ -178,6 +202,9 @@
     <t>1. 在列表中记录一个商品的名称；2. 打开该商品详情页；3. 对比详情页显示的名称与列表名称。</t>
   </si>
   <si>
+    <t>商品列表中显示的商品名称与进入详情页后显示的名称一致。</t>
+  </si>
+  <si>
     <t>TC008</t>
   </si>
   <si>
@@ -193,6 +220,9 @@
     <t>1. 记录列表中某商品的价格；2. 打开该商品详情页；3. 对比两处价格；4. 留意价格格式及是否存在明显异常。</t>
   </si>
   <si>
+    <t>商品列表中显示的商品价格与进入详情页后显示的价格一致。</t>
+  </si>
+  <si>
     <t>TC009</t>
   </si>
   <si>
@@ -208,6 +238,9 @@
     <t>1. 记录数量初始值；2. 点击增加数量；3. 观察数量变化；4. 如允许，尝试减少数量至最小值；5. 记录系统对数量边界的处理。</t>
   </si>
   <si>
+    <t>在商品详情页将 Combination Pliers 的加入数量从 1 改为 2，加入购物车后，商品加入数量及购物车累计数量均符合预期。</t>
+  </si>
+  <si>
     <t>TC010</t>
   </si>
   <si>
@@ -223,6 +256,12 @@
     <t>1. 记录商品名称、单价和选择数量；2. 点击加入购物车；3. 观察页面反馈；4. 打开购物车；5. 核对商品、数量和金额。</t>
   </si>
   <si>
+    <t>点击加入购物车后，页面出现 Oops, something went wrong.，但商品实际加入购物车，数量增加。</t>
+  </si>
+  <si>
+    <t>失败（Fail）</t>
+  </si>
+  <si>
     <t>TC011</t>
   </si>
   <si>
@@ -241,6 +280,9 @@
     <t>1. 记录当前商品列表；2. 选择一个分类；3. 等待列表刷新；4. 检查展示商品是否属于该分类。</t>
   </si>
   <si>
+    <t>勾选 Pliers 分类后，商品列表显示筛选结果；取消勾选后，商品列表恢复为全部商品。</t>
+  </si>
+  <si>
     <t>TC012</t>
   </si>
   <si>
@@ -256,6 +298,9 @@
     <t>1. 选择第一个分类并观察结果；2. 切换到另一个分类；3. 检查列表是否更新；4. 确认结果没有明显残留。</t>
   </si>
   <si>
+    <t>勾选 Hammer 后商品列表发生相应变化；取消后勾选 Wrench，商品列表也相应变化。</t>
+  </si>
+  <si>
     <t>TC013</t>
   </si>
   <si>
@@ -271,6 +316,9 @@
     <t>1. 选择一个商品分类；2. 输入一个与该分类商品相关的关键词并搜索；3. 检查结果是否同时符合关键词和分类条件；4. 若无法组合操作，记录实际限制。</t>
   </si>
   <si>
+    <t>勾选 Pliers 分类并搜索关键词 Pliers 后，最终商品列表同时满足分类筛选和关键词搜索条件。</t>
+  </si>
+  <si>
     <t>TC014</t>
   </si>
   <si>
@@ -286,12 +334,15 @@
     <t>P0</t>
   </si>
   <si>
-    <t>购物车当前为空或已清空；商品列表可访问。</t>
+    <t>购物车为空时添加第一个商品</t>
   </si>
   <si>
     <t>1. 返回商品列表；2. 选择另一个不同的商品；3. 点击加入购物车；4. 记录页面提示；5. 打开购物车，检查第二个商品是否出现及原商品是否保留。</t>
   </si>
   <si>
+    <t>点击加入购物车后，页面出现 Oops, something went wrong.，但商品实际已加入购物车，数量增加。</t>
+  </si>
+  <si>
     <t>TC015</t>
   </si>
   <si>
@@ -322,6 +373,9 @@
     <t>1. 选择一个商品并加入购物车；2. 再次对同一商品执行加入购物车操作；3. 打开购物车；4. 检查该商品是数量增加还是出现重复条目，并记录结果。</t>
   </si>
   <si>
+    <t>再次添加 Combination Pliers 时，页面出现错误提示；返回购物车后，商品数量仍为 2，底部总价仍为 $40.31，未发生变化。</t>
+  </si>
+  <si>
     <t>TC017</t>
   </si>
   <si>
@@ -337,6 +391,9 @@
     <t>1. 记录商品单价、原数量和金额；2. 将数量修改为另一个有效值；3. 确认修改；4. 检查数量、单项金额和购物车总价是否同步更新。</t>
   </si>
   <si>
+    <t>Combination Pliers 数量从 2 改为 1 后，底部总价从 $40.31 变为 $26.16；再改回 2 后，底部总价恢复为 $40.31，均符合预期。</t>
+  </si>
+  <si>
     <t>TC018</t>
   </si>
   <si>
@@ -352,6 +409,9 @@
     <t>1. 记录待删除商品名称及购物车总价；2. 点击该商品对应的删除或移除入口；3. 确认页面变化；4. 检查商品是否消失及总价是否更新。</t>
   </si>
   <si>
+    <t>点击 × 后商品仍在，底部总价不变</t>
+  </si>
+  <si>
     <t>TC019</t>
   </si>
   <si>
@@ -367,6 +427,9 @@
     <t>1. 记录商品单价；2. 记录购物车中该商品数量；3. 记录页面显示的单项 Total；4. 手动计算单价乘数量；5. 对比计算结果与页面金额。</t>
   </si>
   <si>
+    <t>购物车商品行内的 Total 显示 $00.00</t>
+  </si>
+  <si>
     <t>TC020</t>
   </si>
   <si>
@@ -382,6 +445,9 @@
     <t>1. 记录购物车中每个商品的单项金额；2. 将各单项金额相加；3. 记录页面底部显示的总价；4. 对比计算值与页面总价。</t>
   </si>
   <si>
+    <t>$28.30 + $12.01 = $40.31，底部总价正确</t>
+  </si>
+  <si>
     <t>TC021</t>
   </si>
   <si>
@@ -397,6 +463,9 @@
     <t>1. 打开购物车并记录商品及数量；2. 刷新浏览器页面；3. 等待页面加载完成；4. 检查商品、数量和金额是否符合系统设计。</t>
   </si>
   <si>
+    <t>刷新页面后，Combination Pliers 和 Pliers 仍然存在，商品数量及底部总价与刷新前一致。</t>
+  </si>
+  <si>
     <t>TC022</t>
   </si>
   <si>
@@ -412,6 +481,12 @@
     <t>1. 选择一个商品；2. 点击加入购物车；3. 观察是否出现错误提示；4. 若出现提示，检查购物车是否错误增加商品或金额；5. 可刷新后再尝试一次并记录是否复现。</t>
   </si>
   <si>
+    <t>点击加入购物车后出现 Oops, something went wrong.，但商品实际加入购物车，数量增加。该现象在添加不同商品时均有出现。</t>
+  </si>
+  <si>
+    <t>关联 TC010、TC014</t>
+  </si>
+  <si>
     <t>TC023</t>
   </si>
   <si>
@@ -430,6 +505,9 @@
     <t>1. 点击登录入口；2. 等待登录页面加载；3. 检查用户名、密码输入框和提交按钮是否正常显示。</t>
   </si>
   <si>
+    <t>登录页面正常打开，显示邮箱输入框、密码输入框和 Login 按钮，同时显示注册入口及找回密码入口。</t>
+  </si>
+  <si>
     <t>TC024</t>
   </si>
   <si>
@@ -445,6 +523,12 @@
     <t>1. 确保用户名和密码输入框均为空；2. 点击登录按钮；3. 观察页面校验提示和页面状态。</t>
   </si>
   <si>
+    <t>邮箱和密码均为空时，点击 Login，页面显示提示“Invalid email or password”，并停留在登录页面。</t>
+  </si>
+  <si>
+    <t>待判断</t>
+  </si>
+  <si>
     <t>TC025</t>
   </si>
   <si>
@@ -457,6 +541,9 @@
     <t>1. 在用户名输入框输入任意测试用户名；2. 密码框保持为空；3. 点击登录；4. 观察是否提示密码必填或阻止提交。</t>
   </si>
   <si>
+    <t>输入格式正确的测试邮箱 test@example.com，密码留空，点击 Login 后，页面显示“Invalid email or password”，并停留在登录页面。</t>
+  </si>
+  <si>
     <t>TC026</t>
   </si>
   <si>
@@ -472,10 +559,13 @@
     <t>1. 输入无效用户名或错误密码；2. 点击登录；3. 观察登录结果和错误提示；4. 确认页面没有显示为登录成功。</t>
   </si>
   <si>
+    <t>输入测试邮箱 test@example.com 和错误密码 WrongPass123!，点击 Login 后，页面显示“Invalid email or password”，并停留在登录页面。</t>
+  </si>
+  <si>
     <t>TC027</t>
   </si>
   <si>
-    <t>使用有效测试账号登录（具备账号时）</t>
+    <t>注册后使用相同凭据尝试登录</t>
   </si>
   <si>
     <t>登录成功并进入预期状态</t>
@@ -487,6 +577,15 @@
     <t>1. 输入有效测试账号和密码；2. 点击登录；3. 观察页面反馈；4. 检查是否进入登录后的预期状态。</t>
   </si>
   <si>
+    <t>注册提交后未显示明确的成功提示，直接跳转至 My account 页面，右上角显示 User Data not found。退出后使用注册时相同的邮箱和密码登录，提示 Invalid email or password，无法重新登录。</t>
+  </si>
+  <si>
+    <t>已执行，待确认</t>
+  </si>
+  <si>
+    <t>账号是否成功创建尚未确认</t>
+  </si>
+  <si>
     <t>TC028</t>
   </si>
   <si>
@@ -500,6 +599,120 @@
   </si>
   <si>
     <t>1. 修改之前输入的账号或密码；2. 再次点击登录；3. 观察是否允许重试；4. 检查新结果是否与本次输入一致。</t>
+  </si>
+  <si>
+    <t>更换为另一组错误密码后再次点击 Login，页面再次显示“Invalid email or password”，页面未卡住，仍可继续操作。</t>
+  </si>
+  <si>
+    <t>TC029</t>
+  </si>
+  <si>
+    <t>空购物车及购物车入口显示</t>
+  </si>
+  <si>
+    <t>空购物车时页面展示符合设计；添加商品后购物车入口出现，并可以进入购物车</t>
+  </si>
+  <si>
+    <t>未添加商品时页面没有购物车图标；添加商品后图标出现，点击后可以进入购物车</t>
+  </si>
+  <si>
+    <t>1. 打开 With Bugs 版 Toolshop 首页；2. 观察页面顶部是否显示购物车图标；3. 进入商品列表，选择任意商品并打开详情页；4. 点击加入购物车；5. 返回页面顶部，观察购物车图标是否出现；6. 点击购物车图标，检查是否能正常进入购物车页面。</t>
+  </si>
+  <si>
+    <t>空购物车时购物车图标隐藏，是否符合设计需进一步确认。</t>
+  </si>
+  <si>
+    <t>TC030</t>
+  </si>
+  <si>
+    <t>用户注册</t>
+  </si>
+  <si>
+    <t>打开注册页面</t>
+  </si>
+  <si>
+    <t>注册页面正常打开，并显示注册所需的表单字段。</t>
+  </si>
+  <si>
+    <t>已打开 With Bugs 版 Toolshop 网站</t>
+  </si>
+  <si>
+    <t>1. 打开网站首页；2. 点击 Sign in；3. 点击 Register your account；4. 观察注册页面是否正常打开，以及是否显示注册表单。</t>
+  </si>
+  <si>
+    <t>注册页面正常打开，显示 First name、Last name、Date of birth、Address、Postcode、City、Country、State、Phone、E-mail address、Password 等字段，并显示 Register 按钮。</t>
+  </si>
+  <si>
+    <t>TC031</t>
+  </si>
+  <si>
+    <t>购物车商品数量为0时的处理</t>
+  </si>
+  <si>
+    <t>数量为 0 时，系统应合理处理该商品，并保持购物车状态与入口显示一致</t>
+  </si>
+  <si>
+    <t>已打开 With Bugs 版 Toolshop；购物车中存在商品。</t>
+  </si>
+  <si>
+    <t>1. 进入购物车页面；2. 将 Combination Pliers 数量改为0；3. 检查商品行内金额和购物车总价；4. 点击 Proceed to checkout；5. 观察页面跳转；6. 返回商品详情页，观察购物车图标；7. 将数量恢复为1，观察图标是否重新出现。</t>
+  </si>
+  <si>
+    <t>数量为0时，商品行内金额显示$00.00，购物车总价显示$0.00。点击 Proceed to checkout 后进入 Customer login 页面。点击浏览器返回后直接回到商品详情页。进一步观察发现，购物车数量为0时图标消失，无法通过图标进入购物车；多商品场景下，数量为0的商品仍可能留在清单中。将数量恢复为1后，购物车图标重新出现。</t>
+  </si>
+  <si>
+    <t>已执行，待判断</t>
+  </si>
+  <si>
+    <t>TC032</t>
+  </si>
+  <si>
+    <t>购物车商品数量输入负数</t>
+  </si>
+  <si>
+    <t>系统应拒绝负数或自动修正为合法数量；商品数量、行内金额及购物车总价应保持一致。</t>
+  </si>
+  <si>
+    <t>购物车中有商品，商品数量为1，页面总价正常显示。</t>
+  </si>
+  <si>
+    <t>1. 进入购物车页面；2. 将商品数量从1改为-1；3. 按Enter或点击页面空白处；4. 观察数量框和购物车总价；5. 刷新页面；6. 再次观察商品数量。</t>
+  </si>
+  <si>
+    <t>输入-1后，数量框暂时显示-1，但购物车总价没有变化；刷新页面后，商品数量自动恢复为1。</t>
+  </si>
+  <si>
+    <t>TC033</t>
+  </si>
+  <si>
+    <t>购物车商品数量输入小数</t>
+  </si>
+  <si>
+    <t>系统应拒绝非整数数量或自动修正为合法整数；商品数量和总价应保持一致。</t>
+  </si>
+  <si>
+    <t>购物车中有商品，商品数量为1。</t>
+  </si>
+  <si>
+    <t>1. 进入购物车页面；2. 将商品数量从1改为1.5；3. 按Enter或点击页面空白处；4. 观察数量框显示值及购物车总价。</t>
+  </si>
+  <si>
+    <t>输入1.5后，数量自动恢复为1。</t>
+  </si>
+  <si>
+    <t>TC034</t>
+  </si>
+  <si>
+    <t>购物车商品数量输入字母</t>
+  </si>
+  <si>
+    <t>数量输入框应拒绝非数字字符，商品数量和购物车总价不应受到非法输入影响。</t>
+  </si>
+  <si>
+    <t>1. 进入购物车页面；2. 尝试将商品数量输入框的内容改为abc；3. 观察是否能输入字母及商品数量、总价是否变化。</t>
+  </si>
+  <si>
+    <t>尝试输入 abc 后，数量框变为空白，最后金额显示为 0</t>
   </si>
 </sst>
 </file>
@@ -512,7 +725,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -531,13 +744,6 @@
       <sz val="10"/>
       <name val="Microsoft YaHei"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <u/>
@@ -1029,148 +1235,148 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1540,7 +1746,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:K35"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
@@ -1548,12 +1754,13 @@
     <col min="4" max="4" width="42" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
     <col min="6" max="6" width="50.8181818181818" customWidth="1"/>
-    <col min="7" max="7" width="49.1818181818182" customWidth="1"/>
-    <col min="8" max="8" width="29.2727272727273" customWidth="1"/>
+    <col min="7" max="7" width="69.7272727272727" customWidth="1"/>
+    <col min="8" max="8" width="64.6909090909091" customWidth="1"/>
     <col min="9" max="9" width="28.7272727272727" customWidth="1"/>
+    <col min="10" max="10" width="30.6272727272727" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:9">
+    <row r="1" ht="28" customHeight="1" spans="1:10">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1581,765 +1788,1039 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" ht="32" customHeight="1" spans="1:9">
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1" spans="1:10">
       <c r="A2" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" s="2"/>
+    </row>
+    <row r="3" ht="32" customHeight="1" spans="1:10">
+      <c r="A3" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F2" s="4" t="s">
+      <c r="C3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="3" ht="32" customHeight="1" spans="1:9">
-      <c r="A3" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" s="2" t="s">
+      <c r="F3" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="I3" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" ht="32" customHeight="1" spans="1:9">
+      <c r="J3" s="2"/>
+    </row>
+    <row r="4" ht="32" customHeight="1" spans="1:10">
       <c r="A4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="J4" s="2"/>
+    </row>
+    <row r="5" ht="32" customHeight="1" spans="1:10">
+      <c r="A5" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F5" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" ht="32" customHeight="1" spans="1:9">
-      <c r="A5" s="2" t="s">
+      <c r="G5" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J5" s="2"/>
+    </row>
+    <row r="6" ht="32" customHeight="1" spans="1:10">
+      <c r="A6" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J6" s="2"/>
+    </row>
+    <row r="7" ht="32" customHeight="1" spans="1:10">
+      <c r="A7" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J7" s="2"/>
+    </row>
+    <row r="8" ht="32" customHeight="1" spans="1:10">
+      <c r="A8" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J8" s="2"/>
+    </row>
+    <row r="9" ht="32" customHeight="1" spans="1:10">
+      <c r="A9" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J9" s="2"/>
+    </row>
+    <row r="10" ht="32" customHeight="1" spans="1:10">
+      <c r="A10" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J10" s="2"/>
+    </row>
+    <row r="11" ht="32" customHeight="1" spans="1:10">
+      <c r="A11" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="J11" s="2"/>
+    </row>
+    <row r="12" ht="32" customHeight="1" spans="1:10">
+      <c r="A12" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J12" s="2"/>
+    </row>
+    <row r="13" ht="32" customHeight="1" spans="1:10">
+      <c r="A13" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J13" s="2"/>
+    </row>
+    <row r="14" ht="32" customHeight="1" spans="1:10">
+      <c r="A14" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="E14" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" ht="32" customHeight="1" spans="1:9">
-      <c r="A6" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="7" ht="32" customHeight="1" spans="1:9">
-      <c r="A7" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" ht="32" customHeight="1" spans="1:9">
-      <c r="A8" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" ht="32" customHeight="1" spans="1:9">
-      <c r="A9" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="10" ht="32" customHeight="1" spans="1:9">
-      <c r="A10" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="11" ht="32" customHeight="1" spans="1:9">
-      <c r="A11" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="12" ht="32" customHeight="1" spans="1:9">
-      <c r="A12" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="13" ht="32" customHeight="1" spans="1:9">
-      <c r="A13" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F13" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="G13" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="H13" s="4"/>
-      <c r="I13" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="14" ht="32" customHeight="1" spans="1:9">
-      <c r="A14" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="C14" s="2" t="s">
+      <c r="F14" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J14" s="2"/>
+    </row>
+    <row r="15" ht="32" customHeight="1" spans="1:10">
+      <c r="A15" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="I15" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="H14" s="4"/>
-      <c r="I14" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="15" ht="32" customHeight="1" spans="1:9">
-      <c r="A15" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="E15" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="G15" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="H15" s="4"/>
-      <c r="I15" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="16" ht="32" customHeight="1" spans="1:9">
+      <c r="J15" s="2"/>
+    </row>
+    <row r="16" ht="32" customHeight="1" spans="1:10">
       <c r="A16" s="2" t="s">
-        <v>85</v>
+        <v>102</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>86</v>
+        <v>103</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>82</v>
+        <v>98</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="H16" s="4"/>
+        <v>106</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>101</v>
+      </c>
       <c r="I16" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="17" ht="32" customHeight="1" spans="1:9">
+        <v>74</v>
+      </c>
+      <c r="J16" s="2"/>
+    </row>
+    <row r="17" ht="32" customHeight="1" spans="1:11">
       <c r="A17" s="2" t="s">
-        <v>90</v>
+        <v>107</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>91</v>
+        <v>108</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>92</v>
+        <v>109</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="H17" s="4"/>
+        <v>111</v>
+      </c>
+      <c r="H17" s="4" t="s">
+        <v>112</v>
+      </c>
       <c r="I17" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="18" ht="32" customHeight="1" spans="1:9">
+        <v>74</v>
+      </c>
+      <c r="J17" s="2"/>
+    </row>
+    <row r="18" ht="32" customHeight="1" spans="1:11">
       <c r="A18" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="B18" s="2" t="s">
-        <v>79</v>
-      </c>
       <c r="C18" s="2" t="s">
-        <v>96</v>
+        <v>114</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>97</v>
+        <v>115</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>82</v>
+        <v>98</v>
       </c>
       <c r="F18" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="H18" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J18" s="2"/>
+    </row>
+    <row r="19" ht="32" customHeight="1" spans="1:11">
+      <c r="A19" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="E19" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="G18" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="H18" s="4"/>
-      <c r="I18" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="19" ht="32" customHeight="1" spans="1:9">
-      <c r="A19" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="E19" s="6" t="s">
-        <v>82</v>
-      </c>
       <c r="F19" s="4" t="s">
-        <v>103</v>
+        <v>122</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="H19" s="4"/>
+        <v>123</v>
+      </c>
+      <c r="H19" s="4" t="s">
+        <v>124</v>
+      </c>
       <c r="I19" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="20" ht="32" customHeight="1" spans="1:9">
+        <v>74</v>
+      </c>
+      <c r="J19" s="2"/>
+    </row>
+    <row r="20" ht="32" customHeight="1" spans="1:11">
       <c r="A20" s="2" t="s">
-        <v>105</v>
+        <v>125</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>106</v>
+        <v>126</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>107</v>
+        <v>127</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>82</v>
+        <v>98</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>108</v>
+        <v>128</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="H20" s="4"/>
+        <v>129</v>
+      </c>
+      <c r="H20" s="4" t="s">
+        <v>130</v>
+      </c>
       <c r="I20" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="21" ht="32" customHeight="1" spans="1:9">
+        <v>74</v>
+      </c>
+      <c r="J20" s="2"/>
+    </row>
+    <row r="21" ht="32" customHeight="1" spans="1:11">
       <c r="A21" s="2" t="s">
-        <v>110</v>
+        <v>131</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>111</v>
+        <v>132</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>112</v>
+        <v>133</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>82</v>
+        <v>98</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>113</v>
+        <v>134</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="H21" s="4"/>
+        <v>135</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>136</v>
+      </c>
       <c r="I21" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="22" ht="32" customHeight="1" spans="1:9">
+        <v>18</v>
+      </c>
+      <c r="J21" s="2"/>
+    </row>
+    <row r="22" ht="32" customHeight="1" spans="1:11">
       <c r="A22" s="2" t="s">
-        <v>115</v>
+        <v>137</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>116</v>
+        <v>138</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>117</v>
+        <v>139</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>118</v>
+        <v>140</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="H22" s="4"/>
+        <v>141</v>
+      </c>
+      <c r="H22" s="4" t="s">
+        <v>142</v>
+      </c>
       <c r="I22" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="23" ht="32" customHeight="1" spans="1:9">
+        <v>18</v>
+      </c>
+      <c r="J22" s="2"/>
+    </row>
+    <row r="23" ht="32" customHeight="1" spans="1:11">
       <c r="A23" s="2" t="s">
-        <v>120</v>
+        <v>143</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>121</v>
+        <v>144</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>122</v>
+        <v>145</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>82</v>
+        <v>98</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>123</v>
+        <v>146</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="H23" s="4"/>
+        <v>147</v>
+      </c>
+      <c r="H23" s="4" t="s">
+        <v>148</v>
+      </c>
       <c r="I23" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="24" ht="32" customHeight="1" spans="1:9">
+        <v>74</v>
+      </c>
+      <c r="J23" s="2" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="24" ht="32" customHeight="1" spans="1:11">
       <c r="A24" s="2" t="s">
-        <v>125</v>
+        <v>150</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>126</v>
+        <v>151</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>127</v>
+        <v>152</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>128</v>
+        <v>153</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>129</v>
+        <v>154</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="H24" s="4"/>
+        <v>155</v>
+      </c>
+      <c r="H24" s="4" t="s">
+        <v>156</v>
+      </c>
       <c r="I24" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="25" ht="32" customHeight="1" spans="1:9">
+        <v>18</v>
+      </c>
+      <c r="J24" s="2"/>
+    </row>
+    <row r="25" ht="32" customHeight="1" spans="1:11">
       <c r="A25" s="2" t="s">
-        <v>131</v>
+        <v>157</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>126</v>
+        <v>151</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>132</v>
+        <v>158</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>133</v>
+        <v>159</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>134</v>
+        <v>160</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="H25" s="4"/>
+        <v>161</v>
+      </c>
+      <c r="H25" s="4" t="s">
+        <v>162</v>
+      </c>
       <c r="I25" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="26" ht="32" customHeight="1" spans="1:9">
+        <v>163</v>
+      </c>
+      <c r="J25" s="2"/>
+    </row>
+    <row r="26" ht="32" customHeight="1" spans="1:11">
       <c r="A26" s="2" t="s">
-        <v>136</v>
+        <v>164</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>126</v>
+        <v>151</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>137</v>
+        <v>165</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>138</v>
+        <v>166</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>134</v>
+        <v>160</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="H26" s="4"/>
+        <v>167</v>
+      </c>
+      <c r="H26" s="4" t="s">
+        <v>168</v>
+      </c>
       <c r="I26" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="27" ht="32" customHeight="1" spans="1:9">
+        <v>163</v>
+      </c>
+      <c r="J26" s="2"/>
+    </row>
+    <row r="27" ht="32" customHeight="1" spans="1:11">
       <c r="A27" s="2" t="s">
-        <v>140</v>
+        <v>169</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>126</v>
+        <v>151</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>141</v>
+        <v>170</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>142</v>
+        <v>171</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>143</v>
+        <v>172</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="H27" s="4"/>
+        <v>173</v>
+      </c>
+      <c r="H27" s="4" t="s">
+        <v>174</v>
+      </c>
       <c r="I27" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="28" ht="32" customHeight="1" spans="1:9">
+        <v>18</v>
+      </c>
+      <c r="J27" s="2"/>
+    </row>
+    <row r="28" ht="42" customHeight="1" spans="1:11">
       <c r="A28" s="2" t="s">
-        <v>145</v>
+        <v>175</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>126</v>
+        <v>151</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>146</v>
+        <v>176</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>147</v>
+        <v>177</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>148</v>
+        <v>178</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="H28" s="4"/>
+        <v>179</v>
+      </c>
+      <c r="H28" s="4" t="s">
+        <v>180</v>
+      </c>
       <c r="I28" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="29" ht="32" customHeight="1" spans="1:9">
+        <v>181</v>
+      </c>
+      <c r="J28" s="2" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="29" ht="32" customHeight="1" spans="1:11">
       <c r="A29" s="2" t="s">
-        <v>150</v>
+        <v>183</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>126</v>
+        <v>151</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>151</v>
+        <v>184</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>152</v>
+        <v>185</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>153</v>
+        <v>186</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="H29" s="4"/>
+        <v>187</v>
+      </c>
+      <c r="H29" s="4" t="s">
+        <v>188</v>
+      </c>
       <c r="I29" s="2" t="s">
-        <v>16</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="J29" s="2"/>
+    </row>
+    <row r="30" ht="50" customHeight="1" spans="1:11">
+      <c r="A30" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="E30" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="G30" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="H30" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="I30" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J30" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="K30" s="2"/>
+    </row>
+    <row r="31" ht="41" customHeight="1" spans="1:11">
+      <c r="A31" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="E31" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="G31" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="H31" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="I31" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J31" s="2"/>
+    </row>
+    <row r="32" ht="72.5" spans="1:11">
+      <c r="A32" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="G32" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="H32" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="I32" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="J32" s="2"/>
+    </row>
+    <row r="33" ht="29" spans="1:10">
+      <c r="A33" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="G33" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H33" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="I33" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="J33" s="2"/>
+    </row>
+    <row r="34" ht="29" spans="1:10">
+      <c r="A34" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="E34" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="G34" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="H34" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="I34" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J34" s="2"/>
+    </row>
+    <row r="35" ht="29" spans="1:10">
+      <c r="A35" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="E35" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="G35" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="H35" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="I35" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="J35" s="2"/>
     </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:E29" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:E32" etc:filterBottomFollowUsedRange="0">
     <extLst/>
   </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>